<commit_message>
Describe your changes briefly
</commit_message>
<xml_diff>
--- a/clients/FMG 09.22.2025.xlsx
+++ b/clients/FMG 09.22.2025.xlsx
@@ -4973,7 +4973,7 @@
         <v>Oscar</v>
       </c>
       <c r="H2" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I2" t="str">
         <v>02/27/2026</v>
@@ -5002,7 +5002,7 @@
         <v>Oscar</v>
       </c>
       <c r="H3" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I3" t="str">
         <v>02/27/2026</v>
@@ -5031,7 +5031,7 @@
         <v>Oscar</v>
       </c>
       <c r="H4" t="str">
-        <v>Already</v>
+        <v>Need to add demo</v>
       </c>
     </row>
     <row r="5">
@@ -5057,7 +5057,7 @@
         <v>Oscar</v>
       </c>
       <c r="H5" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I5" t="str">
         <v>02/27/2026</v>
@@ -5086,7 +5086,7 @@
         <v>Oscar</v>
       </c>
       <c r="H6" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I6" t="str">
         <v>02/27/2026</v>
@@ -5115,7 +5115,7 @@
         <v>Oscar</v>
       </c>
       <c r="H7" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I7" t="str">
         <v>02/27/2026</v>
@@ -5274,7 +5274,7 @@
         <v>Oscar</v>
       </c>
       <c r="H13" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I13" t="str">
         <v>02/27/2026</v>
@@ -5303,7 +5303,7 @@
         <v>Oscar</v>
       </c>
       <c r="H14" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I14" t="str">
         <v>02/27/2026</v>
@@ -5332,7 +5332,7 @@
         <v>Oscar</v>
       </c>
       <c r="H15" t="str">
-        <v>Already</v>
+        <v>Need to add demo</v>
       </c>
     </row>
     <row r="16">
@@ -5358,7 +5358,7 @@
         <v>Oscar</v>
       </c>
       <c r="H16" t="str">
-        <v>Already</v>
+        <v>Need to add demo</v>
       </c>
     </row>
     <row r="17">
@@ -5384,7 +5384,7 @@
         <v>Oscar</v>
       </c>
       <c r="H17" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I17" t="str">
         <v>02/27/2026</v>
@@ -5491,7 +5491,7 @@
         <v>Oscar</v>
       </c>
       <c r="H21" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I21" t="str">
         <v>02/27/2026</v>
@@ -5520,7 +5520,7 @@
         <v>Oscar</v>
       </c>
       <c r="H22" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I22" t="str">
         <v>02/27/2026</v>
@@ -5549,7 +5549,7 @@
         <v>Oscar</v>
       </c>
       <c r="H23" t="str">
-        <v>Sent</v>
+        <v>Need to add demo</v>
       </c>
       <c r="I23" t="str">
         <v>02/27/2026</v>
@@ -5578,7 +5578,7 @@
         <v>Oscar</v>
       </c>
       <c r="H24" t="str">
-        <v>Already</v>
+        <v>Need to add demo</v>
       </c>
     </row>
   </sheetData>

</xml_diff>